<commit_message>
chore: weekend fixtures spreadsheet (2026-08-17T16:05:32Z)
</commit_message>
<xml_diff>
--- a/downloads/weekend-fixtures-2026-08-22.xlsx
+++ b/downloads/weekend-fixtures-2026-08-22.xlsx
@@ -12273,14 +12273,14 @@
           <t>Fish Hoek</t>
         </is>
       </c>
-      <c r="C215" s="10" t="inlineStr">
-        <is>
-          <t>Away</t>
+      <c r="C215" s="8" t="inlineStr">
+        <is>
+          <t>Home</t>
         </is>
       </c>
       <c r="D215" s="7" t="inlineStr">
         <is>
-          <t>Rygersdal</t>
+          <t>Shosholoza FC</t>
         </is>
       </c>
       <c r="E215" s="7" t="inlineStr">
@@ -12295,7 +12295,7 @@
       </c>
       <c r="G215" s="7" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="H215" s="9" t="inlineStr">
@@ -12305,12 +12305,12 @@
       </c>
       <c r="I215" s="7" t="inlineStr">
         <is>
-          <t>Premier Division</t>
+          <t>4th Division</t>
         </is>
       </c>
       <c r="J215" s="7" t="inlineStr">
         <is>
-          <t>Norway Parks Royal Road A</t>
+          <t>Fish Hoek A</t>
         </is>
       </c>
       <c r="K215" s="6" t="inlineStr"/>
@@ -12328,14 +12328,14 @@
           <t>Fish Hoek</t>
         </is>
       </c>
-      <c r="C216" s="4" t="inlineStr">
-        <is>
-          <t>Home</t>
+      <c r="C216" s="11" t="inlineStr">
+        <is>
+          <t>Away</t>
         </is>
       </c>
       <c r="D216" s="3" t="inlineStr">
         <is>
-          <t>Shosholoza FC</t>
+          <t>Rygersdal</t>
         </is>
       </c>
       <c r="E216" s="3" t="inlineStr">
@@ -12360,12 +12360,12 @@
       </c>
       <c r="I216" s="3" t="inlineStr">
         <is>
-          <t>4th Division</t>
+          <t>Premier Division</t>
         </is>
       </c>
       <c r="J216" s="3" t="inlineStr">
         <is>
-          <t>Fish Hoek A</t>
+          <t>Norway Parks Royal Road A</t>
         </is>
       </c>
       <c r="K216" s="2" t="inlineStr"/>
@@ -27060,14 +27060,14 @@
           <t>Shosholoza FC</t>
         </is>
       </c>
-      <c r="C484" s="4" t="inlineStr">
-        <is>
-          <t>Home</t>
+      <c r="C484" s="11" t="inlineStr">
+        <is>
+          <t>Away</t>
         </is>
       </c>
       <c r="D484" s="3" t="inlineStr">
         <is>
-          <t>Edgemead G/W</t>
+          <t>Fish Hoek</t>
         </is>
       </c>
       <c r="E484" s="3" t="inlineStr">
@@ -27082,7 +27082,7 @@
       </c>
       <c r="G484" s="3" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="H484" s="5" t="inlineStr">
@@ -27092,12 +27092,12 @@
       </c>
       <c r="I484" s="3" t="inlineStr">
         <is>
-          <t>3rd Division</t>
+          <t>4th Division</t>
         </is>
       </c>
       <c r="J484" s="3" t="inlineStr">
         <is>
-          <t>Pelican Heights Sports Ground Pelican A</t>
+          <t>Fish Hoek A</t>
         </is>
       </c>
       <c r="K484" s="2" t="inlineStr"/>
@@ -27115,14 +27115,14 @@
           <t>Shosholoza FC</t>
         </is>
       </c>
-      <c r="C485" s="10" t="inlineStr">
-        <is>
-          <t>Away</t>
+      <c r="C485" s="8" t="inlineStr">
+        <is>
+          <t>Home</t>
         </is>
       </c>
       <c r="D485" s="7" t="inlineStr">
         <is>
-          <t>Fish Hoek</t>
+          <t>Edgemead G/W</t>
         </is>
       </c>
       <c r="E485" s="7" t="inlineStr">
@@ -27147,12 +27147,12 @@
       </c>
       <c r="I485" s="7" t="inlineStr">
         <is>
-          <t>4th Division</t>
+          <t>3rd Division</t>
         </is>
       </c>
       <c r="J485" s="7" t="inlineStr">
         <is>
-          <t>Fish Hoek A</t>
+          <t>Pelican Heights Sports Ground Pelican A</t>
         </is>
       </c>
       <c r="K485" s="6" t="inlineStr"/>
@@ -43027,7 +43027,7 @@
       </c>
       <c r="C216" s="3" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="D216" s="5" t="inlineStr">
@@ -43037,22 +43037,22 @@
       </c>
       <c r="E216" s="3" t="inlineStr">
         <is>
-          <t>Vets 035 B</t>
+          <t>4th Division</t>
         </is>
       </c>
       <c r="F216" s="3" t="inlineStr">
         <is>
-          <t>Everton United</t>
+          <t>Fish Hoek</t>
         </is>
       </c>
       <c r="G216" s="3" t="inlineStr">
         <is>
-          <t>Bellville City</t>
+          <t>Shosholoza FC</t>
         </is>
       </c>
       <c r="H216" s="3" t="inlineStr">
         <is>
-          <t>Heideveld Sports Complex</t>
+          <t>Fish Hoek A</t>
         </is>
       </c>
       <c r="I216" s="2" t="inlineStr"/>
@@ -43082,22 +43082,22 @@
       </c>
       <c r="E217" s="7" t="inlineStr">
         <is>
-          <t>Vets 045 A</t>
+          <t>Vets 035 B</t>
         </is>
       </c>
       <c r="F217" s="7" t="inlineStr">
         <is>
-          <t>Lansdowne</t>
+          <t>Everton United</t>
         </is>
       </c>
       <c r="G217" s="7" t="inlineStr">
         <is>
-          <t>Hanover Park</t>
+          <t>Bellville City</t>
         </is>
       </c>
       <c r="H217" s="7" t="inlineStr">
         <is>
-          <t>Lansdowne Chukker Road A</t>
+          <t>Heideveld Sports Complex</t>
         </is>
       </c>
       <c r="I217" s="6" t="inlineStr"/>
@@ -43132,17 +43132,17 @@
       </c>
       <c r="F218" s="3" t="inlineStr">
         <is>
-          <t>Table View</t>
+          <t>Lansdowne</t>
         </is>
       </c>
       <c r="G218" s="3" t="inlineStr">
         <is>
-          <t>Stephanian Ottery</t>
+          <t>Hanover Park</t>
         </is>
       </c>
       <c r="H218" s="3" t="inlineStr">
         <is>
-          <t>Table View B</t>
+          <t>Lansdowne Chukker Road A</t>
         </is>
       </c>
       <c r="I218" s="2" t="inlineStr"/>
@@ -43172,22 +43172,22 @@
       </c>
       <c r="E219" s="7" t="inlineStr">
         <is>
-          <t>Vets O50 C</t>
+          <t>Vets 045 A</t>
         </is>
       </c>
       <c r="F219" s="7" t="inlineStr">
         <is>
-          <t>West End United C</t>
+          <t>Table View</t>
         </is>
       </c>
       <c r="G219" s="7" t="inlineStr">
         <is>
-          <t>Tramway B</t>
+          <t>Stephanian Ottery</t>
         </is>
       </c>
       <c r="H219" s="7" t="inlineStr">
         <is>
-          <t>West End United West End Park B</t>
+          <t>Table View B</t>
         </is>
       </c>
       <c r="I219" s="6" t="inlineStr"/>
@@ -43207,7 +43207,7 @@
       </c>
       <c r="C220" s="3" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="D220" s="5" t="inlineStr">
@@ -43217,22 +43217,22 @@
       </c>
       <c r="E220" s="3" t="inlineStr">
         <is>
-          <t>3rd Division</t>
+          <t>Vets O50 C</t>
         </is>
       </c>
       <c r="F220" s="3" t="inlineStr">
         <is>
-          <t>Bellville City FC</t>
+          <t>West End United C</t>
         </is>
       </c>
       <c r="G220" s="3" t="inlineStr">
         <is>
-          <t>Bothasig</t>
+          <t>Tramway B</t>
         </is>
       </c>
       <c r="H220" s="3" t="inlineStr">
         <is>
-          <t>Bellville City PP Smit Stadium C</t>
+          <t>West End United West End Park B</t>
         </is>
       </c>
       <c r="I220" s="2" t="inlineStr"/>
@@ -43267,17 +43267,17 @@
       </c>
       <c r="F221" s="7" t="inlineStr">
         <is>
-          <t>Shosholoza FC</t>
+          <t>Bellville City FC</t>
         </is>
       </c>
       <c r="G221" s="7" t="inlineStr">
         <is>
-          <t>Edgemead G/W</t>
+          <t>Bothasig</t>
         </is>
       </c>
       <c r="H221" s="7" t="inlineStr">
         <is>
-          <t>Pelican Heights Sports Ground Pelican A</t>
+          <t>Bellville City PP Smit Stadium C</t>
         </is>
       </c>
       <c r="I221" s="6" t="inlineStr"/>
@@ -43307,22 +43307,22 @@
       </c>
       <c r="E222" s="3" t="inlineStr">
         <is>
-          <t>4th Division</t>
+          <t>3rd Division</t>
         </is>
       </c>
       <c r="F222" s="3" t="inlineStr">
         <is>
-          <t>Fish Hoek</t>
+          <t>Shosholoza FC</t>
         </is>
       </c>
       <c r="G222" s="3" t="inlineStr">
         <is>
-          <t>Shosholoza FC</t>
+          <t>Edgemead G/W</t>
         </is>
       </c>
       <c r="H222" s="3" t="inlineStr">
         <is>
-          <t>Fish Hoek A</t>
+          <t>Pelican Heights Sports Ground Pelican A</t>
         </is>
       </c>
       <c r="I222" s="2" t="inlineStr"/>

</xml_diff>